<commit_message>
fix: complete Arthur validation tests
</commit_message>
<xml_diff>
--- a/07_PlanoTeste_v4.xlsx
+++ b/07_PlanoTeste_v4.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>Arthur</t>
   </si>
@@ -317,6 +317,15 @@
   </si>
   <si>
     <t>Aprovado - o formulario possui campos obrigatorios e, com dados obrigatorios ausentes, a validacao impede o envio.</t>
+  </si>
+  <si>
+    <t>Aprovado - o campo nome agora exige no minimo 3 caracteres no navegador e no backend; "Jo" foi rejeitado.</t>
+  </si>
+  <si>
+    <t>Aprovado - a descricao agora possui limite maxlength de 500 caracteres no formulario e e truncada para 500 no backend.</t>
+  </si>
+  <si>
+    <t>Aprovado - o backend limita a descricao a 500 caracteres antes de gravar no banco, mesmo que a requisicao ignore o formulario.</t>
   </si>
 </sst>
 </file>
@@ -794,7 +803,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="J3" s="7"/>
     </row>
@@ -860,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J6" s="8"/>
     </row>
@@ -878,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="J7" s="7"/>
     </row>

</xml_diff>